<commit_message>
Deck cleanup: remove CallRpt/LTV, promote Zelle, add ARCU→JHBI slide
PPTX changes:
- Remove Call Report AI and Account Opening LTV detail slides
- Zelle Memo Intelligence moved to first position in app detail order
- Add "NOW" launch badge to Zelle Memo card on Portfolio Overview
- Remove Next Steps closing slide
- Move Pricing Tiers to appendix (with divider slide)
- Add ARCU & JHAKnow → JHBI four-quarter migration slide (Fall 2026 launch)
  with CU and Bank track cards, pricing continuity callout, presenter notes
- Market Opportunity: update third segment (remove CallRpt AI framing)
- ROI table: remove Call Report AI and Account Opening LTV rows
- Per-App Pricing: remove those two rows, update total to six apps ~$6.3K/mo
- Revenue Expansion NOW module: updated to Zelle Memo Intelligence

Excel fix:
- B7 (Bank Share of Base) corrected to =1-B6 (was referencing B5)
- Rebuild confirms 0 errors across 208 formulas

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/JHBI_Revenue_Model.xlsx
+++ b/JHBI_Revenue_Model.xlsx
@@ -1801,8 +1801,8 @@
         <v>60</v>
       </c>
       <c r="B7" s="29" t="n">
-        <f aca="false">1-B5</f>
-        <v>-1659</v>
+        <f aca="false">1-B6</f>
+        <v>0.56</v>
       </c>
       <c r="G7" s="27" t="s">
         <v>61</v>
@@ -2143,19 +2143,19 @@
       </c>
       <c r="B30" s="38" t="n">
         <f aca="false">Assumptions!B22*(1-$B$7)</f>
-        <v>8300000</v>
+        <v>2200</v>
       </c>
       <c r="C30" s="38" t="n">
         <f aca="false">Assumptions!C22*(1-$B$7)</f>
-        <v>13280000</v>
+        <v>3520</v>
       </c>
       <c r="D30" s="38" t="n">
         <f aca="false">Assumptions!D22*(1-$B$7)</f>
-        <v>24900000</v>
+        <v>6600</v>
       </c>
       <c r="E30" s="38" t="n">
         <f aca="false">Assumptions!E22*(1-$B$7)</f>
-        <v>41500000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2165,19 +2165,19 @@
       </c>
       <c r="B31" s="40" t="n">
         <f aca="false">Assumptions!B23*(1-$B$7)</f>
-        <v>13280000</v>
+        <v>3520</v>
       </c>
       <c r="C31" s="40" t="n">
         <f aca="false">Assumptions!C23*(1-$B$7)</f>
-        <v>19920000</v>
+        <v>5280</v>
       </c>
       <c r="D31" s="40" t="n">
         <f aca="false">Assumptions!D23*(1-$B$7)</f>
-        <v>36520000</v>
+        <v>9680</v>
       </c>
       <c r="E31" s="40" t="n">
         <f aca="false">Assumptions!E23*(1-$B$7)</f>
-        <v>58100000</v>
+        <v>15400</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2187,19 +2187,19 @@
       </c>
       <c r="B32" s="38" t="n">
         <f aca="false">Assumptions!B24*(1-$B$7)</f>
-        <v>9960000</v>
+        <v>2640</v>
       </c>
       <c r="C32" s="38" t="n">
         <f aca="false">Assumptions!C24*(1-$B$7)</f>
-        <v>16600000</v>
+        <v>4400</v>
       </c>
       <c r="D32" s="38" t="n">
         <f aca="false">Assumptions!D24*(1-$B$7)</f>
-        <v>29880000</v>
+        <v>7920</v>
       </c>
       <c r="E32" s="38" t="n">
         <f aca="false">Assumptions!E24*(1-$B$7)</f>
-        <v>46480000</v>
+        <v>12320</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2209,19 +2209,19 @@
       </c>
       <c r="B33" s="40" t="n">
         <f aca="false">Assumptions!B25*(1-$B$7)</f>
-        <v>13280000</v>
+        <v>3520</v>
       </c>
       <c r="C33" s="40" t="n">
         <f aca="false">Assumptions!C25*(1-$B$7)</f>
-        <v>19920000</v>
+        <v>5280</v>
       </c>
       <c r="D33" s="40" t="n">
         <f aca="false">Assumptions!D25*(1-$B$7)</f>
-        <v>33200000</v>
+        <v>8800</v>
       </c>
       <c r="E33" s="40" t="n">
         <f aca="false">Assumptions!E25*(1-$B$7)</f>
-        <v>49800000</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2231,19 +2231,19 @@
       </c>
       <c r="B34" s="38" t="n">
         <f aca="false">Assumptions!B26*(1-$B$7)</f>
-        <v>13280000</v>
+        <v>3520</v>
       </c>
       <c r="C34" s="38" t="n">
         <f aca="false">Assumptions!C26*(1-$B$7)</f>
-        <v>24900000</v>
+        <v>6600</v>
       </c>
       <c r="D34" s="38" t="n">
         <f aca="false">Assumptions!D26*(1-$B$7)</f>
-        <v>41500000</v>
+        <v>11000</v>
       </c>
       <c r="E34" s="38" t="n">
         <f aca="false">Assumptions!E26*(1-$B$7)</f>
-        <v>66400000</v>
+        <v>17600</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>